<commit_message>
Cleaned dimensions multi-links for sector coupled
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" firstSheet="1" activeTab="7"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="IntermittentUnitBlock" sheetId="1" r:id="rId1"/>
@@ -457,9 +457,6 @@
     <t>ID of the hyperarch - sector coupled only</t>
   </si>
   <si>
-    <t>[NB]</t>
-  </si>
-  <si>
     <t>HyperArcID</t>
   </si>
   <si>
@@ -497,6 +494,9 @@
   </si>
   <si>
     <t>Marginal cost of the line</t>
+  </si>
+  <si>
+    <t>[L] | [NB]</t>
   </si>
 </sst>
 </file>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>7</v>
@@ -1948,10 +1948,10 @@
     </row>
     <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -1968,10 +1968,10 @@
     </row>
     <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
@@ -2542,7 +2542,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -2562,7 +2562,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -2582,7 +2582,7 @@
         <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>10</v>
@@ -2602,7 +2602,7 @@
         <v>13</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>10</v>
@@ -2613,16 +2613,16 @@
         <v>138</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>10</v>
@@ -2630,7 +2630,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>25</v>
@@ -2642,7 +2642,7 @@
         <v>13</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -2662,7 +2662,7 @@
         <v>13</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>10</v>
@@ -2801,7 +2801,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -2821,7 +2821,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -2901,7 +2901,7 @@
         <v>13</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>142</v>
@@ -2921,7 +2921,7 @@
         <v>13</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>32</v>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>7</v>
@@ -2997,7 +2997,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -3017,7 +3017,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -3097,7 +3097,7 @@
         <v>13</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -3105,10 +3105,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>7</v>
@@ -3125,7 +3125,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>142</v>
@@ -3137,7 +3137,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Preprocessing of capital cost 0 generators
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
   </bookViews>
   <sheets>
     <sheet name="IntermittentUnitBlock" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="165">
   <si>
     <t>Name</t>
   </si>
@@ -509,6 +509,18 @@
   </si>
   <si>
     <t>Ramp in shut t</t>
+  </si>
+  <si>
+    <t>MinGeneration</t>
+  </si>
+  <si>
+    <t>Minimum generation over time horizon</t>
+  </si>
+  <si>
+    <t>MaxGeneration</t>
+  </si>
+  <si>
+    <t>Maximum generation over time horizon</t>
   </si>
 </sst>
 </file>
@@ -878,7 +890,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" style="2" bestFit="1" customWidth="1"/>
@@ -1086,6 +1098,46 @@
         <v>1</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Included standing losses for sector coupled
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="IntermittentUnitBlock" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="167">
   <si>
     <t>Name</t>
   </si>
@@ -521,6 +521,12 @@
   </si>
   <si>
     <t>Maximum generation over time horizon</t>
+  </si>
+  <si>
+    <t>StandingBatteryRho</t>
+  </si>
+  <si>
+    <t>Standing losses</t>
   </si>
 </sst>
 </file>
@@ -1593,7 +1599,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.44140625" style="2" bestFit="1" customWidth="1"/>
@@ -1796,10 +1802,10 @@
     </row>
     <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>93</v>
+        <v>165</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>93</v>
+        <v>166</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>7</v>
@@ -1807,20 +1813,19 @@
       <c r="D10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>94</v>
+      <c r="E10" s="3">
+        <v>1</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>7</v>
@@ -1829,19 +1834,19 @@
         <v>13</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" s="5"/>
+        <v>32</v>
+      </c>
+      <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>7</v>
@@ -1859,10 +1864,10 @@
     </row>
     <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
@@ -1874,16 +1879,16 @@
         <v>20</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
@@ -1901,10 +1906,10 @@
     </row>
     <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
@@ -1912,22 +1917,20 @@
       <c r="D15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="3">
-        <v>1</v>
+      <c r="E15" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>105</v>
-      </c>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
@@ -1947,10 +1950,10 @@
     </row>
     <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
@@ -1958,20 +1961,22 @@
       <c r="D17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="3" t="s">
-        <v>20</v>
+      <c r="E17" s="3">
+        <v>1</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G17" s="5"/>
+      <c r="G17" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
@@ -1979,8 +1984,8 @@
       <c r="D18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="3">
-        <v>1</v>
+      <c r="E18" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>32</v>
@@ -1989,10 +1994,10 @@
     </row>
     <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
@@ -2010,10 +2015,10 @@
     </row>
     <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>7</v>
@@ -2031,10 +2036,10 @@
     </row>
     <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
@@ -2052,10 +2057,10 @@
     </row>
     <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>149</v>
+        <v>116</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -2069,13 +2074,14 @@
       <c r="F22" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="G22" s="5"/>
     </row>
     <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
@@ -2087,6 +2093,26 @@
         <v>1</v>
       </c>
       <c r="F23" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>